<commit_message>
Makro: taquillas efecto madera y antracita en los 6 paises
- 10 filas nuevas en cada offer_template (ES, PT, IT, FR, DE, NL): precio de
  Espana del maestro sin el IVA del pais, stock 0, almacen/plazo/Shipping Group y
  descuentos por cantidad con las reglas de la web (scripts/anadir-madera-makro.ts).
- makro.ts reconoce los sufijos _M/_A y los colores Madera/Antracita del CSV.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/Makro/offer_template DE.xlsx
+++ b/public/plantillas/Makro/offer_template DE.xlsx
@@ -2232,34 +2232,514 @@
       </c>
     </row>
     <row r="38" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G38" s="3"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641534</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F38">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3">
+        <v>100.84</v>
+      </c>
+      <c r="H38">
+        <v>1</v>
+      </c>
+      <c r="I38">
+        <v>2</v>
+      </c>
+      <c r="L38" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M38" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N38">
+        <v>97.81</v>
+      </c>
+      <c r="O38">
+        <v>96.81</v>
+      </c>
+      <c r="P38">
+        <v>95.8</v>
+      </c>
+      <c r="Q38">
+        <v>94.79</v>
+      </c>
+      <c r="V38" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SMALL</t>
+        </is>
+      </c>
     </row>
     <row r="39" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G39" s="3"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641480</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F39">
+        <v>0</v>
+      </c>
+      <c r="G39" s="3">
+        <v>100</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39">
+        <v>2</v>
+      </c>
+      <c r="L39" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M39" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N39">
+        <v>97</v>
+      </c>
+      <c r="O39">
+        <v>96</v>
+      </c>
+      <c r="P39">
+        <v>95</v>
+      </c>
+      <c r="Q39">
+        <v>94</v>
+      </c>
+      <c r="V39" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SMALL</t>
+        </is>
+      </c>
     </row>
     <row r="40" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G40" s="3"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641497</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F40">
+        <v>0</v>
+      </c>
+      <c r="G40" s="3">
+        <v>252.1</v>
+      </c>
+      <c r="H40">
+        <v>1</v>
+      </c>
+      <c r="I40">
+        <v>2</v>
+      </c>
+      <c r="L40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N40">
+        <v>244.54</v>
+      </c>
+      <c r="O40">
+        <v>242.02</v>
+      </c>
+      <c r="P40">
+        <v>239.49</v>
+      </c>
+      <c r="Q40">
+        <v>236.97</v>
+      </c>
+      <c r="V40" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LARGE</t>
+        </is>
+      </c>
     </row>
     <row r="41" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G41" s="3"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641442</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41" s="3">
+        <v>252.1</v>
+      </c>
+      <c r="H41">
+        <v>1</v>
+      </c>
+      <c r="I41">
+        <v>2</v>
+      </c>
+      <c r="L41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N41">
+        <v>244.54</v>
+      </c>
+      <c r="O41">
+        <v>242.02</v>
+      </c>
+      <c r="P41">
+        <v>239.49</v>
+      </c>
+      <c r="Q41">
+        <v>236.97</v>
+      </c>
+      <c r="V41" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LARGE</t>
+        </is>
+      </c>
     </row>
     <row r="42" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G42" s="3"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641503</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42" s="3">
+        <v>150.42</v>
+      </c>
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42">
+        <v>2</v>
+      </c>
+      <c r="L42" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M42" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N42">
+        <v>145.91</v>
+      </c>
+      <c r="O42">
+        <v>144.4</v>
+      </c>
+      <c r="P42">
+        <v>142.9</v>
+      </c>
+      <c r="Q42">
+        <v>141.39</v>
+      </c>
+      <c r="V42" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="43" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G43" s="3"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641459</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43" s="3">
+        <v>150.42</v>
+      </c>
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43">
+        <v>2</v>
+      </c>
+      <c r="L43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N43">
+        <v>145.91</v>
+      </c>
+      <c r="O43">
+        <v>144.4</v>
+      </c>
+      <c r="P43">
+        <v>142.9</v>
+      </c>
+      <c r="Q43">
+        <v>141.39</v>
+      </c>
+      <c r="V43" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="44" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G44" s="3"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641510</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F44">
+        <v>0</v>
+      </c>
+      <c r="G44" s="3">
+        <v>167.23</v>
+      </c>
+      <c r="H44">
+        <v>1</v>
+      </c>
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="L44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N44">
+        <v>162.21</v>
+      </c>
+      <c r="O44">
+        <v>160.54</v>
+      </c>
+      <c r="P44">
+        <v>158.87</v>
+      </c>
+      <c r="Q44">
+        <v>157.2</v>
+      </c>
+      <c r="V44" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="45" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G45" s="3"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641466</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45" s="3">
+        <v>168.07</v>
+      </c>
+      <c r="H45">
+        <v>1</v>
+      </c>
+      <c r="I45">
+        <v>2</v>
+      </c>
+      <c r="L45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N45">
+        <v>163.03</v>
+      </c>
+      <c r="O45">
+        <v>161.35</v>
+      </c>
+      <c r="P45">
+        <v>159.67</v>
+      </c>
+      <c r="Q45">
+        <v>157.99</v>
+      </c>
+      <c r="V45" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIUM</t>
+        </is>
+      </c>
     </row>
     <row r="46" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G46" s="3"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641527</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46" s="3">
+        <v>234.45</v>
+      </c>
+      <c r="H46">
+        <v>1</v>
+      </c>
+      <c r="I46">
+        <v>2</v>
+      </c>
+      <c r="L46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N46">
+        <v>227.42</v>
+      </c>
+      <c r="O46">
+        <v>225.07</v>
+      </c>
+      <c r="P46">
+        <v>222.73</v>
+      </c>
+      <c r="Q46">
+        <v>220.38</v>
+      </c>
+      <c r="V46" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LARGE</t>
+        </is>
+      </c>
     </row>
     <row r="47" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="G47" s="3"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8437027641473</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TwinThink</t>
+        </is>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47" s="3">
+        <v>234.45</v>
+      </c>
+      <c r="H47">
+        <v>1</v>
+      </c>
+      <c r="I47">
+        <v>2</v>
+      </c>
+      <c r="L47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DE_MAIN</t>
+        </is>
+      </c>
+      <c r="M47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FR_MAIN</t>
+        </is>
+      </c>
+      <c r="N47">
+        <v>227.42</v>
+      </c>
+      <c r="O47">
+        <v>225.07</v>
+      </c>
+      <c r="P47">
+        <v>222.73</v>
+      </c>
+      <c r="Q47">
+        <v>220.38</v>
+      </c>
+      <c r="V47" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LARGE</t>
+        </is>
+      </c>
     </row>
     <row r="48" spans="7:7" ht="15.5" x14ac:dyDescent="0.35">
       <c r="G48" s="3"/>

</xml_diff>